<commit_message>
NumMethods: passed lw9, lw10, lw11 and completed the course
</commit_message>
<xml_diff>
--- a/Numerical methods/LW10/LW10.xlsx
+++ b/Numerical methods/LW10/LW10.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\studies\Numerical methods\LW10\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\studies\Numerical methods\LW10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD50A948-FD0A-48E4-87BB-1019F14B3227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE51DA06-E5E3-4AB7-B058-F4547936AFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3030" yWindow="1320" windowWidth="21585" windowHeight="11370" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Формула трапеций" sheetId="1" r:id="rId1"/>
@@ -30,9 +30,6 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -421,9 +418,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:I7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.35">
       <c r="E2" t="s">
         <v>2</v>
       </c>
@@ -431,7 +428,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>0</v>
       </c>
@@ -452,7 +449,7 @@
         <v>-1.7435390549999998</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>1</v>
       </c>
@@ -466,7 +463,7 @@
         <v>-0.96227569000000002</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.35">
       <c r="E5">
         <v>0.5</v>
       </c>
@@ -474,7 +471,7 @@
         <v>5.6035939999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>6</v>
       </c>
@@ -488,7 +485,7 @@
         <v>0.62822496999999999</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>5</v>
       </c>
@@ -510,13 +507,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A5CF17-ACA1-4576-8D1D-229A7AE8905F}">
   <dimension ref="B2:M150"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="12" max="12" width="10.140625" customWidth="1"/>
+    <col min="12" max="12" width="10.1796875" customWidth="1"/>
     <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -524,7 +521,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -532,7 +529,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.35">
       <c r="H5" t="s">
         <v>2</v>
       </c>
@@ -543,7 +540,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.35">
       <c r="E6" t="s">
         <v>6</v>
       </c>
@@ -568,7 +565,7 @@
         <v>-1.3411741911111099</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.35">
       <c r="E7" t="s">
         <v>7</v>
       </c>
@@ -587,7 +584,7 @@
         <v>-9.8405409600000002</v>
       </c>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.35">
       <c r="E8" t="s">
         <v>5</v>
       </c>
@@ -605,7 +602,7 @@
         <v>-2.3356408000000002</v>
       </c>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.35">
       <c r="H9">
         <v>0</v>
       </c>
@@ -617,7 +614,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.35">
       <c r="H10">
         <v>0.33333332999999998</v>
       </c>
@@ -629,7 +626,7 @@
         <v>-0.19382002000000001</v>
       </c>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.35">
       <c r="H11">
         <v>0.66666667000000002</v>
       </c>
@@ -641,7 +638,7 @@
         <v>0.76707787999999999</v>
       </c>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
       <c r="H12">
         <v>1</v>
       </c>
@@ -653,7 +650,7 @@
         <v>0.8811213</v>
       </c>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.35">
       <c r="H13">
         <v>1.3333333300000001</v>
       </c>
@@ -665,7 +662,7 @@
         <v>2.7754694799999999</v>
       </c>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.35">
       <c r="H14">
         <v>1.6666666699999999</v>
       </c>
@@ -677,7 +674,7 @@
         <v>1.9691733199999999</v>
       </c>
     </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:13" x14ac:dyDescent="0.35">
       <c r="H15">
         <v>2</v>
       </c>
@@ -689,7 +686,7 @@
         <v>1.34315574</v>
       </c>
     </row>
-    <row r="17" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H17" t="s">
         <v>2</v>
       </c>
@@ -700,7 +697,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="5:13" x14ac:dyDescent="0.35">
       <c r="E18" t="s">
         <v>9</v>
       </c>
@@ -726,7 +723,7 @@
         <v>-1.2057642155555544</v>
       </c>
     </row>
-    <row r="19" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H19">
         <v>-0.83333332999999998</v>
       </c>
@@ -738,7 +735,7 @@
         <v>-14.438247240000001</v>
       </c>
     </row>
-    <row r="20" spans="5:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="5:13" ht="29" x14ac:dyDescent="0.35">
       <c r="H20">
         <v>-0.66666667000000002</v>
       </c>
@@ -757,7 +754,7 @@
         <v>9.0273317037037042E-3</v>
       </c>
     </row>
-    <row r="21" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H21">
         <v>-0.5</v>
       </c>
@@ -769,7 +766,7 @@
         <v>-6.7885117199999998</v>
       </c>
     </row>
-    <row r="22" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H22">
         <v>-0.33333332999999998</v>
       </c>
@@ -781,7 +778,7 @@
         <v>-2.3356408000000002</v>
       </c>
     </row>
-    <row r="23" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H23">
         <v>-0.16666666999999999</v>
       </c>
@@ -793,7 +790,7 @@
         <v>-3.1439441600000002</v>
       </c>
     </row>
-    <row r="24" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H24">
         <v>0</v>
       </c>
@@ -805,7 +802,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="25" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H25">
         <v>0.16666666999999999</v>
       </c>
@@ -817,7 +814,7 @@
         <v>-1.1096278799999999</v>
       </c>
     </row>
-    <row r="26" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H26">
         <v>0.33333332999999998</v>
       </c>
@@ -829,7 +826,7 @@
         <v>-0.19382002000000001</v>
       </c>
     </row>
-    <row r="27" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H27">
         <v>0.5</v>
       </c>
@@ -841,7 +838,7 @@
         <v>0.22414376</v>
       </c>
     </row>
-    <row r="28" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H28">
         <v>0.66666667000000002</v>
       </c>
@@ -853,7 +850,7 @@
         <v>0.38353893999999999</v>
       </c>
     </row>
-    <row r="29" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H29">
         <v>0.83333332999999998</v>
       </c>
@@ -865,7 +862,7 @@
         <v>1.2718319199999999</v>
       </c>
     </row>
-    <row r="30" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H30">
         <v>1</v>
       </c>
@@ -877,7 +874,7 @@
         <v>0.8811213</v>
       </c>
     </row>
-    <row r="31" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H31">
         <v>1.1666666699999999</v>
       </c>
@@ -889,7 +886,7 @@
         <v>2.25782404</v>
       </c>
     </row>
-    <row r="32" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H32">
         <v>1.3333333300000001</v>
       </c>
@@ -901,7 +898,7 @@
         <v>1.38773474</v>
       </c>
     </row>
-    <row r="33" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H33">
         <v>1.5</v>
       </c>
@@ -913,7 +910,7 @@
         <v>3.3306569600000002</v>
       </c>
     </row>
-    <row r="34" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H34">
         <v>1.6666666699999999</v>
       </c>
@@ -925,7 +922,7 @@
         <v>1.9691733199999999</v>
       </c>
     </row>
-    <row r="35" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H35">
         <v>1.8333333300000001</v>
       </c>
@@ -937,7 +934,7 @@
         <v>4.6136893600000004</v>
       </c>
     </row>
-    <row r="36" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H36">
         <v>2</v>
       </c>
@@ -949,7 +946,7 @@
         <v>1.34315574</v>
       </c>
     </row>
-    <row r="38" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H38" t="s">
         <v>2</v>
       </c>
@@ -960,7 +957,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="5:13" x14ac:dyDescent="0.35">
       <c r="E39" t="s">
         <v>5</v>
       </c>
@@ -986,7 +983,7 @@
         <v>-1.2051102377777758</v>
       </c>
     </row>
-    <row r="40" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H40">
         <v>-0.91666667000000002</v>
       </c>
@@ -998,7 +995,7 @@
         <v>-17.644587319999999</v>
       </c>
     </row>
-    <row r="41" spans="5:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="5:13" ht="29" x14ac:dyDescent="0.35">
       <c r="H41">
         <v>-0.83333332999999998</v>
       </c>
@@ -1017,7 +1014,7 @@
         <v>4.359851851856907E-5</v>
       </c>
     </row>
-    <row r="42" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H42">
         <v>-0.75</v>
       </c>
@@ -1029,7 +1026,7 @@
         <v>-11.891605520000001</v>
       </c>
     </row>
-    <row r="43" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H43">
         <v>-0.66666667000000002</v>
       </c>
@@ -1041,7 +1038,7 @@
         <v>-4.9202704800000001</v>
       </c>
     </row>
-    <row r="44" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H44">
         <v>-0.58333332999999998</v>
       </c>
@@ -1053,7 +1050,7 @@
         <v>-8.1679518800000004</v>
       </c>
     </row>
-    <row r="45" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H45">
         <v>-0.5</v>
       </c>
@@ -1065,7 +1062,7 @@
         <v>-3.3942558599999999</v>
       </c>
     </row>
-    <row r="46" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H46">
         <v>-0.41666667000000002</v>
       </c>
@@ -1077,7 +1074,7 @@
         <v>-5.63888532</v>
       </c>
     </row>
-    <row r="47" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H47">
         <v>-0.33333332999999998</v>
       </c>
@@ -1089,7 +1086,7 @@
         <v>-2.3356408000000002</v>
       </c>
     </row>
-    <row r="48" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H48">
         <v>-0.25</v>
       </c>
@@ -1101,7 +1098,7 @@
         <v>-3.8491027600000001</v>
       </c>
     </row>
-    <row r="49" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H49">
         <v>-0.16666666999999999</v>
       </c>
@@ -1113,7 +1110,7 @@
         <v>-1.5719720800000001</v>
       </c>
     </row>
-    <row r="50" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H50">
         <v>-8.3333329999999997E-2</v>
       </c>
@@ -1125,7 +1122,7 @@
         <v>-2.5334883600000002</v>
       </c>
     </row>
-    <row r="51" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H51">
         <v>0</v>
       </c>
@@ -1137,7 +1134,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="52" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H52">
         <v>8.3333329999999997E-2</v>
       </c>
@@ -1149,7 +1146,7 @@
         <v>-1.5292332399999999</v>
       </c>
     </row>
-    <row r="53" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H53">
         <v>0.16666666999999999</v>
       </c>
@@ -1161,7 +1158,7 @@
         <v>-0.55481393999999995</v>
       </c>
     </row>
-    <row r="54" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H54">
         <v>0.25</v>
       </c>
@@ -1173,7 +1170,7 @@
         <v>-0.73171023999999996</v>
       </c>
     </row>
-    <row r="55" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H55">
         <v>0.33333332999999998</v>
       </c>
@@ -1185,7 +1182,7 @@
         <v>-0.19382002000000001</v>
       </c>
     </row>
-    <row r="56" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H56">
         <v>0.41666667000000002</v>
       </c>
@@ -1197,7 +1194,7 @@
         <v>-7.0865360000000002E-2</v>
       </c>
     </row>
-    <row r="57" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H57">
         <v>0.5</v>
       </c>
@@ -1209,7 +1206,7 @@
         <v>0.11207188</v>
       </c>
     </row>
-    <row r="58" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H58">
         <v>0.58333332999999998</v>
       </c>
@@ -1221,7 +1218,7 @@
         <v>0.50210312000000001</v>
       </c>
     </row>
-    <row r="59" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H59">
         <v>0.66666667000000002</v>
       </c>
@@ -1233,7 +1230,7 @@
         <v>0.38353893999999999</v>
       </c>
     </row>
-    <row r="60" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H60">
         <v>0.75</v>
       </c>
@@ -1245,7 +1242,7 @@
         <v>1.0226118</v>
       </c>
     </row>
-    <row r="61" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H61">
         <v>0.83333332999999998</v>
       </c>
@@ -1257,7 +1254,7 @@
         <v>0.63591595999999995</v>
       </c>
     </row>
-    <row r="62" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H62">
         <v>0.91666667000000002</v>
       </c>
@@ -1269,7 +1266,7 @@
         <v>1.5175322</v>
       </c>
     </row>
-    <row r="63" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H63">
         <v>1</v>
       </c>
@@ -1281,7 +1278,7 @@
         <v>0.8811213</v>
       </c>
     </row>
-    <row r="64" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H64">
         <v>1.0833333300000001</v>
       </c>
@@ -1293,7 +1290,7 @@
         <v>2.0082857199999999</v>
       </c>
     </row>
-    <row r="65" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H65">
         <v>1.1666666699999999</v>
       </c>
@@ -1305,7 +1302,7 @@
         <v>1.12891202</v>
       </c>
     </row>
-    <row r="66" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H66">
         <v>1.25</v>
       </c>
@@ -1317,7 +1314,7 @@
         <v>2.51289988</v>
       </c>
     </row>
-    <row r="67" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H67">
         <v>1.3333333300000001</v>
       </c>
@@ -1329,7 +1326,7 @@
         <v>1.38773474</v>
       </c>
     </row>
-    <row r="68" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="68" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H68">
         <v>1.4166666699999999</v>
       </c>
@@ -1341,7 +1338,7 @@
         <v>3.0474323600000002</v>
       </c>
     </row>
-    <row r="69" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H69">
         <v>1.5</v>
       </c>
@@ -1353,7 +1350,7 @@
         <v>1.6653284800000001</v>
       </c>
     </row>
-    <row r="70" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H70">
         <v>1.5833333300000001</v>
       </c>
@@ -1365,7 +1362,7 @@
         <v>3.6270039600000001</v>
       </c>
     </row>
-    <row r="71" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H71">
         <v>1.6666666699999999</v>
       </c>
@@ -1377,7 +1374,7 @@
         <v>1.9691733199999999</v>
       </c>
     </row>
-    <row r="72" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H72">
         <v>1.75</v>
       </c>
@@ -1389,7 +1386,7 @@
         <v>4.2665902000000004</v>
       </c>
     </row>
-    <row r="73" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="73" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H73">
         <v>1.8333333300000001</v>
       </c>
@@ -1401,7 +1398,7 @@
         <v>2.3068446800000002</v>
       </c>
     </row>
-    <row r="74" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="74" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H74">
         <v>1.9166666699999999</v>
       </c>
@@ -1413,7 +1410,7 @@
         <v>4.9816656000000004</v>
       </c>
     </row>
-    <row r="75" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="75" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H75">
         <v>2</v>
       </c>
@@ -1425,7 +1422,7 @@
         <v>1.34315574</v>
       </c>
     </row>
-    <row r="77" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H77" t="s">
         <v>2</v>
       </c>
@@ -1436,7 +1433,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="78" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="78" spans="5:13" x14ac:dyDescent="0.35">
       <c r="E78" t="s">
         <v>5</v>
       </c>
@@ -1462,7 +1459,7 @@
         <v>-1.205066401944443</v>
       </c>
     </row>
-    <row r="79" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="79" spans="5:13" x14ac:dyDescent="0.35">
       <c r="H79">
         <v>-0.95833332999999998</v>
       </c>
@@ -1474,7 +1471,7 @@
         <v>-19.565027879999999</v>
       </c>
     </row>
-    <row r="80" spans="5:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="80" spans="5:13" ht="29" x14ac:dyDescent="0.35">
       <c r="H80">
         <v>-0.91666667000000002</v>
       </c>
@@ -1493,7 +1490,7 @@
         <v>2.9223888888522491E-6</v>
       </c>
     </row>
-    <row r="81" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H81">
         <v>-0.875</v>
       </c>
@@ -1505,7 +1502,7 @@
         <v>-15.94627872</v>
       </c>
     </row>
-    <row r="82" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H82">
         <v>-0.83333332999999998</v>
       </c>
@@ -1517,7 +1514,7 @@
         <v>-7.2191236200000004</v>
       </c>
     </row>
-    <row r="83" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H83">
         <v>-0.79166667000000002</v>
       </c>
@@ -1529,7 +1526,7 @@
         <v>-13.094053199999999</v>
       </c>
     </row>
-    <row r="84" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H84">
         <v>-0.75</v>
       </c>
@@ -1541,7 +1538,7 @@
         <v>-5.9458027600000003</v>
       </c>
     </row>
-    <row r="85" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H85">
         <v>-0.70833332999999998</v>
       </c>
@@ -1553,7 +1550,7 @@
         <v>-10.8123346</v>
       </c>
     </row>
-    <row r="86" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H86">
         <v>-0.66666667000000002</v>
       </c>
@@ -1565,7 +1562,7 @@
         <v>-4.9202704800000001</v>
       </c>
     </row>
-    <row r="87" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H87">
         <v>-0.625</v>
       </c>
@@ -1577,7 +1574,7 @@
         <v>-8.9628797200000001</v>
       </c>
     </row>
-    <row r="88" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H88">
         <v>-0.58333332999999998</v>
       </c>
@@ -1589,7 +1586,7 @@
         <v>-4.0839759400000002</v>
       </c>
     </row>
-    <row r="89" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H89">
         <v>-0.54166667000000002</v>
       </c>
@@ -1601,7 +1598,7 @@
         <v>-7.4459740400000003</v>
       </c>
     </row>
-    <row r="90" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H90">
         <v>-0.5</v>
       </c>
@@ -1613,7 +1610,7 @@
         <v>-3.3942558599999999</v>
       </c>
     </row>
-    <row r="91" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H91">
         <v>-0.45833332999999998</v>
       </c>
@@ -1625,7 +1622,7 @@
         <v>-6.1882639599999996</v>
       </c>
     </row>
-    <row r="92" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H92">
         <v>-0.41666667000000002</v>
       </c>
@@ -1637,7 +1634,7 @@
         <v>-2.81944266</v>
       </c>
     </row>
-    <row r="93" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H93">
         <v>-0.375</v>
       </c>
@@ -1649,7 +1646,7 @@
         <v>-5.1348399200000001</v>
       </c>
     </row>
-    <row r="94" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H94">
         <v>-0.33333332999999998</v>
       </c>
@@ -1661,7 +1658,7 @@
         <v>-2.3356408000000002</v>
       </c>
     </row>
-    <row r="95" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H95">
         <v>-0.29166667000000002</v>
       </c>
@@ -1673,7 +1670,7 @@
         <v>-4.2439532800000004</v>
       </c>
     </row>
-    <row r="96" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H96">
         <v>-0.25</v>
       </c>
@@ -1685,7 +1682,7 @@
         <v>-1.92455138</v>
       </c>
     </row>
-    <row r="97" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H97">
         <v>-0.20833333000000001</v>
       </c>
@@ -1697,7 +1694,7 @@
         <v>-3.4834133600000001</v>
       </c>
     </row>
-    <row r="98" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H98">
         <v>-0.16666666999999999</v>
       </c>
@@ -1709,7 +1706,7 @@
         <v>-1.5719720800000001</v>
       </c>
     </row>
-    <row r="99" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H99">
         <v>-0.125</v>
       </c>
@@ -1721,7 +1718,7 @@
         <v>-2.8280797999999998</v>
       </c>
     </row>
-    <row r="100" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H100">
         <v>-8.3333329999999997E-2</v>
       </c>
@@ -1733,7 +1730,7 @@
         <v>-1.2667441800000001</v>
       </c>
     </row>
-    <row r="101" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H101">
         <v>-4.1666670000000003E-2</v>
       </c>
@@ -1745,7 +1742,7 @@
         <v>-2.25808484</v>
       </c>
     </row>
-    <row r="102" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H102">
         <v>0</v>
       </c>
@@ -1757,7 +1754,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="103" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H103">
         <v>4.1666670000000003E-2</v>
       </c>
@@ -1769,7 +1766,7 @@
         <v>-1.7575539600000001</v>
       </c>
     </row>
-    <row r="104" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H104">
         <v>8.3333329999999997E-2</v>
       </c>
@@ -1781,7 +1778,7 @@
         <v>-0.76461661999999997</v>
       </c>
     </row>
-    <row r="105" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H105">
         <v>0.125</v>
       </c>
@@ -1793,7 +1790,7 @@
         <v>-1.3136704800000001</v>
       </c>
     </row>
-    <row r="106" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H106">
         <v>0.16666666999999999</v>
       </c>
@@ -1805,7 +1802,7 @@
         <v>-0.55481393999999995</v>
       </c>
     </row>
-    <row r="107" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H107">
         <v>0.20833333000000001</v>
       </c>
@@ -1817,7 +1814,7 @@
         <v>-0.91598195999999998</v>
       </c>
     </row>
-    <row r="108" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H108">
         <v>0.25</v>
       </c>
@@ -1829,7 +1826,7 @@
         <v>-0.36585511999999998</v>
       </c>
     </row>
-    <row r="109" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H109">
         <v>0.29166667000000002</v>
       </c>
@@ -1841,7 +1838,7 @@
         <v>-0.55588040000000005</v>
       </c>
     </row>
-    <row r="110" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H110">
         <v>0.33333332999999998</v>
       </c>
@@ -1853,7 +1850,7 @@
         <v>-0.19382002000000001</v>
       </c>
     </row>
-    <row r="111" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H111">
         <v>0.375</v>
       </c>
@@ -1865,7 +1862,7 @@
         <v>-0.22620763999999999</v>
       </c>
     </row>
-    <row r="112" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H112">
         <v>0.41666667000000002</v>
       </c>
@@ -1877,7 +1874,7 @@
         <v>-3.5432680000000001E-2</v>
       </c>
     </row>
-    <row r="113" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H113">
         <v>0.45833332999999998</v>
       </c>
@@ -1889,7 +1886,7 @@
         <v>7.9048160000000006E-2</v>
       </c>
     </row>
-    <row r="114" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H114">
         <v>0.5</v>
       </c>
@@ -1901,7 +1898,7 @@
         <v>0.11207188</v>
       </c>
     </row>
-    <row r="115" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H115">
         <v>0.54166667000000002</v>
       </c>
@@ -1913,7 +1910,7 @@
         <v>0.36498700000000001</v>
       </c>
     </row>
-    <row r="116" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H116">
         <v>0.58333332999999998</v>
       </c>
@@ -1925,7 +1922,7 @@
         <v>0.25105156000000001</v>
       </c>
     </row>
-    <row r="117" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="117" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H117">
         <v>0.625</v>
       </c>
@@ -1937,7 +1934,7 @@
         <v>0.63598120000000002</v>
       </c>
     </row>
-    <row r="118" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H118">
         <v>0.66666667000000002</v>
       </c>
@@ -1949,7 +1946,7 @@
         <v>0.38353893999999999</v>
       </c>
     </row>
-    <row r="119" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="119" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H119">
         <v>0.70833332999999998</v>
       </c>
@@ -1961,7 +1958,7 @@
         <v>0.89582079999999997</v>
       </c>
     </row>
-    <row r="120" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="120" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H120">
         <v>0.75</v>
       </c>
@@ -1973,7 +1970,7 @@
         <v>0.51130589999999998</v>
       </c>
     </row>
-    <row r="121" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="121" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H121">
         <v>0.79166667000000002</v>
       </c>
@@ -1985,7 +1982,7 @@
         <v>1.1478295599999999</v>
       </c>
     </row>
-    <row r="122" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H122">
         <v>0.83333332999999998</v>
       </c>
@@ -1997,7 +1994,7 @@
         <v>0.63591595999999995</v>
       </c>
     </row>
-    <row r="123" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H123">
         <v>0.875</v>
       </c>
@@ -2009,7 +2006,7 @@
         <v>1.3949584399999999</v>
       </c>
     </row>
-    <row r="124" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H124">
         <v>0.91666667000000002</v>
       </c>
@@ -2021,7 +2018,7 @@
         <v>0.7587661</v>
       </c>
     </row>
-    <row r="125" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="125" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H125">
         <v>0.95833332999999998</v>
       </c>
@@ -2033,7 +2030,7 @@
         <v>1.6398617200000001</v>
       </c>
     </row>
-    <row r="126" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="126" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H126">
         <v>1</v>
       </c>
@@ -2045,7 +2042,7 @@
         <v>0.8811213</v>
       </c>
     </row>
-    <row r="127" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="127" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H127">
         <v>1.0416666699999999</v>
       </c>
@@ -2057,7 +2054,7 @@
         <v>1.8849591999999999</v>
       </c>
     </row>
-    <row r="128" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="128" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H128">
         <v>1.0833333300000001</v>
       </c>
@@ -2069,7 +2066,7 @@
         <v>1.00414286</v>
       </c>
     </row>
-    <row r="129" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="129" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H129">
         <v>1.125</v>
       </c>
@@ -2081,7 +2078,7 @@
         <v>2.13248792</v>
       </c>
     </row>
-    <row r="130" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="130" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H130">
         <v>1.1666666699999999</v>
       </c>
@@ -2093,7 +2090,7 @@
         <v>1.12891202</v>
       </c>
     </row>
-    <row r="131" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H131">
         <v>1.2083333300000001</v>
       </c>
@@ -2105,7 +2102,7 @@
         <v>2.3845458399999999</v>
       </c>
     </row>
-    <row r="132" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="132" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H132">
         <v>1.25</v>
       </c>
@@ -2117,7 +2114,7 @@
         <v>1.25644994</v>
       </c>
     </row>
-    <row r="133" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="133" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H133">
         <v>1.2916666699999999</v>
       </c>
@@ -2129,7 +2126,7 @@
         <v>2.6431282399999998</v>
       </c>
     </row>
-    <row r="134" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="134" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H134">
         <v>1.3333333300000001</v>
       </c>
@@ -2141,7 +2138,7 @@
         <v>1.38773474</v>
       </c>
     </row>
-    <row r="135" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="135" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H135">
         <v>1.375</v>
       </c>
@@ -2153,7 +2150,7 @@
         <v>2.9101595200000001</v>
       </c>
     </row>
-    <row r="136" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="136" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H136">
         <v>1.4166666699999999</v>
       </c>
@@ -2165,7 +2162,7 @@
         <v>1.5237161800000001</v>
       </c>
     </row>
-    <row r="137" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="137" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H137">
         <v>1.4583333300000001</v>
       </c>
@@ -2177,7 +2174,7 @@
         <v>3.18752068</v>
       </c>
     </row>
-    <row r="138" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="138" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H138">
         <v>1.5</v>
       </c>
@@ -2189,7 +2186,7 @@
         <v>1.6653284800000001</v>
       </c>
     </row>
-    <row r="139" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="139" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H139">
         <v>1.5416666699999999</v>
       </c>
@@ -2201,7 +2198,7 @@
         <v>3.47707364</v>
       </c>
     </row>
-    <row r="140" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="140" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H140">
         <v>1.5833333300000001</v>
       </c>
@@ -2213,7 +2210,7 @@
         <v>1.8135019800000001</v>
       </c>
     </row>
-    <row r="141" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="141" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H141">
         <v>1.625</v>
       </c>
@@ -2225,7 +2222,7 @@
         <v>3.7806827200000002</v>
       </c>
     </row>
-    <row r="142" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="142" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H142">
         <v>1.6666666699999999</v>
       </c>
@@ -2237,7 +2234,7 @@
         <v>1.9691733199999999</v>
       </c>
     </row>
-    <row r="143" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="143" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H143">
         <v>1.7083333300000001</v>
       </c>
@@ -2249,7 +2246,7 @@
         <v>4.1002349999999996</v>
       </c>
     </row>
-    <row r="144" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="144" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H144">
         <v>1.75</v>
       </c>
@@ -2261,7 +2258,7 @@
         <v>2.1332951000000002</v>
       </c>
     </row>
-    <row r="145" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="145" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H145">
         <v>1.7916666699999999</v>
       </c>
@@ -2273,7 +2270,7 @@
         <v>4.43765828</v>
       </c>
     </row>
-    <row r="146" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="146" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H146">
         <v>1.8333333300000001</v>
       </c>
@@ -2285,7 +2282,7 @@
         <v>2.3068446800000002</v>
       </c>
     </row>
-    <row r="147" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="147" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H147">
         <v>1.875</v>
       </c>
@@ -2297,7 +2294,7 @@
         <v>4.7949384799999999</v>
       </c>
     </row>
-    <row r="148" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="148" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H148">
         <v>1.9166666699999999</v>
       </c>
@@ -2309,7 +2306,7 @@
         <v>2.4908328000000002</v>
       </c>
     </row>
-    <row r="149" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="149" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H149">
         <v>1.9583333300000001</v>
       </c>
@@ -2321,7 +2318,7 @@
         <v>5.1741364000000001</v>
       </c>
     </row>
-    <row r="150" spans="8:10" x14ac:dyDescent="0.25">
+    <row r="150" spans="8:10" x14ac:dyDescent="0.35">
       <c r="H150">
         <v>2</v>
       </c>
@@ -2341,13 +2338,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9F130B2-949E-4FA2-B3CE-F779D2ED1D9B}">
   <dimension ref="B2:M16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="12" max="12" width="11.42578125" customWidth="1"/>
-    <col min="13" max="13" width="14.140625" customWidth="1"/>
+    <col min="12" max="12" width="11.453125" customWidth="1"/>
+    <col min="13" max="13" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -2355,7 +2352,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -2363,7 +2360,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.35">
       <c r="E5" t="s">
         <v>11</v>
       </c>
@@ -2383,7 +2380,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.35">
       <c r="E6">
         <v>1</v>
       </c>
@@ -2412,7 +2409,7 @@
         <v>-1.2050604239493115</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.35">
       <c r="E7">
         <v>2</v>
       </c>
@@ -2434,7 +2431,7 @@
         <v>-0.58321329867052252</v>
       </c>
     </row>
-    <row r="8" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="E8">
         <v>3</v>
       </c>
@@ -2462,7 +2459,7 @@
         <v>-1.205066401944443</v>
       </c>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.35">
       <c r="E9">
         <v>4</v>
       </c>
@@ -2485,7 +2482,7 @@
       </c>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.35">
       <c r="E10">
         <v>5</v>
       </c>
@@ -2508,7 +2505,7 @@
       </c>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.35">
       <c r="E11">
         <v>6</v>
       </c>
@@ -2531,7 +2528,7 @@
       </c>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
       <c r="E12">
         <v>7</v>
       </c>
@@ -2554,7 +2551,7 @@
       </c>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.35">
       <c r="E13">
         <v>8</v>
       </c>
@@ -2577,13 +2574,13 @@
       </c>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.35">
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:13" x14ac:dyDescent="0.35">
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:13" x14ac:dyDescent="0.35">
       <c r="K16" s="2"/>
     </row>
   </sheetData>

</xml_diff>